<commit_message>
JIRA-789 Added retry mechanism and framework enhancements
</commit_message>
<xml_diff>
--- a/testData/Opencart_LoginData.xlsx
+++ b/testData/Opencart_LoginData.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9303"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="225" windowWidth="20730" windowHeight="11760"/>
+    <workbookView xWindow="0" yWindow="2445" windowWidth="19770" windowHeight="7215"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>username</t>
   </si>
@@ -82,6 +83,9 @@
   </si>
   <si>
     <t>Tztejas@13</t>
+  </si>
+  <si>
+    <t>valid</t>
   </si>
 </sst>
 </file>
@@ -489,7 +493,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -535,7 +539,7 @@
         <v>7</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="20.65" x14ac:dyDescent="0.55000000000000004">
@@ -546,7 +550,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="21" x14ac:dyDescent="0.35">

</xml_diff>